<commit_message>
Homologia persisteente y pipeline mas robusto
</commit_message>
<xml_diff>
--- a/Resultados/mapper_nodos.xlsx
+++ b/Resultados/mapper_nodos.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,122 +517,122 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cube0_cluster0</t>
+          <t>cube3_cluster0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>466</v>
+        <v>181</v>
       </c>
       <c r="C2" t="n">
-        <v>229</v>
+        <v>66</v>
       </c>
       <c r="D2" t="n">
-        <v>217</v>
+        <v>67</v>
       </c>
       <c r="E2" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="F2" t="n">
-        <v>49.1</v>
+        <v>36.5</v>
       </c>
       <c r="G2" t="n">
-        <v>46.6</v>
+        <v>37</v>
       </c>
       <c r="H2" t="n">
-        <v>4.3</v>
+        <v>26.5</v>
       </c>
       <c r="I2" t="n">
-        <v>1.1333</v>
+        <v>2.0095</v>
       </c>
       <c r="J2" t="n">
-        <v>33.7203</v>
+        <v>31.4145</v>
       </c>
       <c r="K2" t="n">
-        <v>5.0322</v>
+        <v>5.2376</v>
       </c>
       <c r="L2" t="n">
-        <v>1.5494</v>
+        <v>1.0552</v>
       </c>
       <c r="M2" t="n">
-        <v>6.0107</v>
+        <v>9.348100000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>10.3964</v>
+        <v>10.3215</v>
       </c>
       <c r="O2" t="n">
-        <v>4.0159</v>
+        <v>4.0348</v>
       </c>
       <c r="P2" t="n">
         <v>2</v>
       </c>
       <c r="Q2" t="n">
-        <v>3338.8906</v>
+        <v>3247.5193</v>
       </c>
       <c r="R2" t="n">
-        <v>38.5515</v>
+        <v>38.2494</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cube0_cluster2</t>
+          <t>cube2_cluster0</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>116</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>75</v>
+        <v>38.8</v>
       </c>
       <c r="G3" t="n">
-        <v>25</v>
+        <v>35.3</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>25.9</v>
       </c>
       <c r="I3" t="n">
-        <v>1.165</v>
+        <v>2.0361</v>
       </c>
       <c r="J3" t="n">
-        <v>34.5</v>
+        <v>33.6467</v>
       </c>
       <c r="K3" t="n">
-        <v>3.75</v>
+        <v>5.2328</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>1.9397</v>
       </c>
       <c r="M3" t="n">
-        <v>11.25</v>
+        <v>11.0345</v>
       </c>
       <c r="N3" t="n">
-        <v>7.625</v>
+        <v>10.4172</v>
       </c>
       <c r="O3" t="n">
-        <v>2.9159</v>
+        <v>4.0287</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>3550</v>
+        <v>3316.4224</v>
       </c>
       <c r="R3" t="n">
-        <v>38.5714</v>
+        <v>38.1219</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -643,59 +643,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cube1_cluster2</t>
+          <t>cube4_cluster0</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>36.7</v>
       </c>
       <c r="G4" t="n">
-        <v>25</v>
+        <v>33.5</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>29.8</v>
       </c>
       <c r="I4" t="n">
-        <v>1.165</v>
+        <v>2.1689</v>
       </c>
       <c r="J4" t="n">
-        <v>34.5</v>
+        <v>33.4739</v>
       </c>
       <c r="K4" t="n">
-        <v>3.75</v>
+        <v>5.5349</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>1.0047</v>
       </c>
       <c r="M4" t="n">
-        <v>11.25</v>
+        <v>8.1023</v>
       </c>
       <c r="N4" t="n">
-        <v>7.625</v>
+        <v>10.7805</v>
       </c>
       <c r="O4" t="n">
-        <v>2.9159</v>
+        <v>4.1899</v>
       </c>
       <c r="P4" t="n">
         <v>2</v>
       </c>
       <c r="Q4" t="n">
-        <v>3550</v>
+        <v>3291.8698</v>
       </c>
       <c r="R4" t="n">
-        <v>38.5714</v>
+        <v>38.4611</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -706,59 +706,59 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cube0_cluster1</t>
+          <t>cube34_cluster0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>458</v>
+        <v>148</v>
       </c>
       <c r="C5" t="n">
-        <v>216</v>
+        <v>52</v>
       </c>
       <c r="D5" t="n">
-        <v>224</v>
+        <v>54</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="F5" t="n">
-        <v>47.2</v>
+        <v>35.1</v>
       </c>
       <c r="G5" t="n">
-        <v>48.9</v>
+        <v>36.5</v>
       </c>
       <c r="H5" t="n">
-        <v>3.9</v>
+        <v>28.4</v>
       </c>
       <c r="I5" t="n">
-        <v>1.1708</v>
+        <v>2.1801</v>
       </c>
       <c r="J5" t="n">
-        <v>33.5938</v>
+        <v>31.7635</v>
       </c>
       <c r="K5" t="n">
-        <v>5.024</v>
+        <v>3.9662</v>
       </c>
       <c r="L5" t="n">
-        <v>1.5633</v>
+        <v>1.3108</v>
       </c>
       <c r="M5" t="n">
-        <v>6.1485</v>
+        <v>1.7297</v>
       </c>
       <c r="N5" t="n">
-        <v>10.3836</v>
+        <v>11.7676</v>
       </c>
       <c r="O5" t="n">
-        <v>4.0102</v>
+        <v>4.5915</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>3311.9891</v>
+        <v>3188.8716</v>
       </c>
       <c r="R5" t="n">
-        <v>38.4885</v>
+        <v>38.2915</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -769,628 +769,2203 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cube1_cluster1</t>
+          <t>cube13_cluster0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>405</v>
+        <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>153</v>
+        <v>29</v>
       </c>
       <c r="D6" t="n">
-        <v>223</v>
+        <v>22</v>
       </c>
       <c r="E6" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F6" t="n">
-        <v>37.8</v>
+        <v>39.2</v>
       </c>
       <c r="G6" t="n">
-        <v>55.1</v>
+        <v>29.7</v>
       </c>
       <c r="H6" t="n">
-        <v>7.2</v>
+        <v>31.1</v>
       </c>
       <c r="I6" t="n">
-        <v>1.329</v>
+        <v>2.1868</v>
       </c>
       <c r="J6" t="n">
-        <v>33.3926</v>
+        <v>34.0946</v>
       </c>
       <c r="K6" t="n">
-        <v>4.963</v>
+        <v>4.1892</v>
       </c>
       <c r="L6" t="n">
-        <v>1.5605</v>
+        <v>2.027</v>
       </c>
       <c r="M6" t="n">
-        <v>6.0691</v>
+        <v>1.5676</v>
       </c>
       <c r="N6" t="n">
-        <v>10.6153</v>
+        <v>9.0054</v>
       </c>
       <c r="O6" t="n">
-        <v>4.1113</v>
+        <v>3.4188</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>3338.4864</v>
+        <v>3423.2703</v>
       </c>
       <c r="R6" t="n">
-        <v>38.528</v>
+        <v>38.6042</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cube1_cluster0</t>
+          <t>cube8_cluster0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>402</v>
+        <v>202</v>
       </c>
       <c r="C7" t="n">
-        <v>149</v>
+        <v>77</v>
       </c>
       <c r="D7" t="n">
-        <v>217</v>
+        <v>64</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="F7" t="n">
-        <v>37.1</v>
+        <v>38.1</v>
       </c>
       <c r="G7" t="n">
-        <v>54</v>
+        <v>31.7</v>
       </c>
       <c r="H7" t="n">
-        <v>9</v>
+        <v>30.2</v>
       </c>
       <c r="I7" t="n">
-        <v>1.3585</v>
+        <v>2.2396</v>
       </c>
       <c r="J7" t="n">
-        <v>33.7032</v>
+        <v>34.1734</v>
       </c>
       <c r="K7" t="n">
-        <v>4.9975</v>
+        <v>4.6139</v>
       </c>
       <c r="L7" t="n">
-        <v>1.5622</v>
+        <v>1.9604</v>
       </c>
       <c r="M7" t="n">
-        <v>5.7985</v>
+        <v>6.0594</v>
       </c>
       <c r="N7" t="n">
-        <v>10.6005</v>
+        <v>9.089600000000001</v>
       </c>
       <c r="O7" t="n">
-        <v>4.1021</v>
+        <v>3.4864</v>
       </c>
       <c r="P7" t="n">
         <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>3340.3831</v>
+        <v>3217</v>
       </c>
       <c r="R7" t="n">
-        <v>38.5593</v>
+        <v>38.0106</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cube2_cluster0</t>
+          <t>cube17_cluster0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>46</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>99</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>34.8</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H8" t="n">
-        <v>100</v>
+        <v>28.3</v>
       </c>
       <c r="I8" t="n">
-        <v>4.8625</v>
+        <v>2.2534</v>
       </c>
       <c r="J8" t="n">
-        <v>36.0404</v>
+        <v>27.587</v>
       </c>
       <c r="K8" t="n">
-        <v>5.2828</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
-        <v>1.7172</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>4.8283</v>
+        <v>1.8043</v>
       </c>
       <c r="N8" t="n">
-        <v>10.701</v>
+        <v>11.8565</v>
       </c>
       <c r="O8" t="n">
-        <v>4.1344</v>
+        <v>4.6131</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>3337.2323</v>
+        <v>3392.7391</v>
       </c>
       <c r="R8" t="n">
-        <v>38.3838</v>
+        <v>39.1957</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cube2_cluster1</t>
+          <t>cube38_cluster0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>116</v>
+        <v>75</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E9" t="n">
-        <v>116</v>
+        <v>23</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>29.3</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H9" t="n">
-        <v>100</v>
+        <v>30.7</v>
       </c>
       <c r="I9" t="n">
-        <v>4.8834</v>
+        <v>2.3027</v>
       </c>
       <c r="J9" t="n">
-        <v>35.4827</v>
+        <v>30.2933</v>
       </c>
       <c r="K9" t="n">
-        <v>5.2241</v>
+        <v>6.12</v>
       </c>
       <c r="L9" t="n">
-        <v>1.7328</v>
+        <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>6.6638</v>
+        <v>7.3733</v>
       </c>
       <c r="N9" t="n">
-        <v>10.0655</v>
+        <v>11.616</v>
       </c>
       <c r="O9" t="n">
-        <v>3.8874</v>
+        <v>4.5237</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>3303.6293</v>
+        <v>3356.6</v>
       </c>
       <c r="R9" t="n">
-        <v>38.3793</v>
+        <v>39.1067</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cube3_cluster1</t>
+          <t>cube10_cluster0</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="E10" t="n">
-        <v>194</v>
+        <v>65</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>31.6</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>37.3</v>
       </c>
       <c r="H10" t="n">
-        <v>100</v>
+        <v>31.1</v>
       </c>
       <c r="I10" t="n">
-        <v>5.3673</v>
+        <v>2.3334</v>
       </c>
       <c r="J10" t="n">
-        <v>35.3754</v>
+        <v>32.2057</v>
       </c>
       <c r="K10" t="n">
-        <v>5.1495</v>
+        <v>4.2249</v>
       </c>
       <c r="L10" t="n">
-        <v>1.6598</v>
+        <v>1.0048</v>
       </c>
       <c r="M10" t="n">
-        <v>6.5619</v>
+        <v>4.9809</v>
       </c>
       <c r="N10" t="n">
-        <v>10.0954</v>
+        <v>12.2856</v>
       </c>
       <c r="O10" t="n">
-        <v>3.8761</v>
+        <v>4.7478</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>3314.8814</v>
+        <v>3317.4976</v>
       </c>
       <c r="R10" t="n">
-        <v>38.3829</v>
+        <v>38.7403</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cube3_cluster0</t>
+          <t>cube9_cluster0</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E11" t="n">
-        <v>167</v>
+        <v>64</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>36.6</v>
       </c>
       <c r="H11" t="n">
-        <v>100</v>
+        <v>31.2</v>
       </c>
       <c r="I11" t="n">
-        <v>5.395</v>
+        <v>2.3401</v>
       </c>
       <c r="J11" t="n">
-        <v>35.2218</v>
+        <v>33.2395</v>
       </c>
       <c r="K11" t="n">
-        <v>5.1078</v>
+        <v>4.3805</v>
       </c>
       <c r="L11" t="n">
-        <v>1.6287</v>
+        <v>1.0878</v>
       </c>
       <c r="M11" t="n">
-        <v>5.2575</v>
+        <v>5.7854</v>
       </c>
       <c r="N11" t="n">
-        <v>10.3377</v>
+        <v>10.8849</v>
       </c>
       <c r="O11" t="n">
-        <v>3.9783</v>
+        <v>4.2127</v>
       </c>
       <c r="P11" t="n">
         <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>3333.4192</v>
+        <v>3114.0585</v>
       </c>
       <c r="R11" t="n">
-        <v>38.3584</v>
+        <v>38.0801</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cube4_cluster1</t>
+          <t>cube11_cluster0</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E12" t="n">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>35.1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>31.6</v>
       </c>
       <c r="H12" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="I12" t="n">
-        <v>5.7266</v>
+        <v>2.3604</v>
       </c>
       <c r="J12" t="n">
-        <v>34.3965</v>
+        <v>29.8246</v>
       </c>
       <c r="K12" t="n">
-        <v>5.0147</v>
+        <v>4.2632</v>
       </c>
       <c r="L12" t="n">
-        <v>1.4559</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>5.4706</v>
+        <v>3.1754</v>
       </c>
       <c r="N12" t="n">
-        <v>10.4426</v>
+        <v>12.4719</v>
       </c>
       <c r="O12" t="n">
-        <v>3.9753</v>
+        <v>4.7852</v>
       </c>
       <c r="P12" t="n">
         <v>2</v>
       </c>
       <c r="Q12" t="n">
-        <v>3391.5441</v>
+        <v>3353.0877</v>
       </c>
       <c r="R12" t="n">
-        <v>38.4874</v>
+        <v>38.99</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cube4_cluster0</t>
+          <t>cube7_cluster0</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>84</v>
+        <v>250</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="E13" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>36.4</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>29.6</v>
       </c>
       <c r="H13" t="n">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="I13" t="n">
-        <v>5.8082</v>
+        <v>2.3818</v>
       </c>
       <c r="J13" t="n">
-        <v>34.8788</v>
+        <v>35.2388</v>
       </c>
       <c r="K13" t="n">
-        <v>5.119</v>
+        <v>5.156</v>
       </c>
       <c r="L13" t="n">
-        <v>1.5</v>
+        <v>2.328</v>
       </c>
       <c r="M13" t="n">
-        <v>6.1071</v>
+        <v>6.356</v>
       </c>
       <c r="N13" t="n">
-        <v>10.6238</v>
+        <v>9.808</v>
       </c>
       <c r="O13" t="n">
-        <v>4.0457</v>
+        <v>3.7637</v>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" t="n">
-        <v>3354.0595</v>
+        <v>3432.412</v>
       </c>
       <c r="R13" t="n">
-        <v>38.3401</v>
+        <v>38.3617</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cube4_cluster2</t>
+          <t>cube35_cluster0</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>183</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>30.6</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>35.5</v>
       </c>
       <c r="H14" t="n">
-        <v>100</v>
+        <v>33.9</v>
       </c>
       <c r="I14" t="n">
-        <v>6.3767</v>
+        <v>2.3947</v>
       </c>
       <c r="J14" t="n">
-        <v>33</v>
+        <v>32.3224</v>
       </c>
       <c r="K14" t="n">
-        <v>4</v>
+        <v>4.0328</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>1.0164</v>
       </c>
       <c r="M14" t="n">
-        <v>9.666700000000001</v>
+        <v>3.8087</v>
       </c>
       <c r="N14" t="n">
-        <v>5.6667</v>
+        <v>10.465</v>
       </c>
       <c r="O14" t="n">
-        <v>2.2738</v>
+        <v>4.0936</v>
       </c>
       <c r="P14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>3393.3333</v>
+        <v>3285.4809</v>
       </c>
       <c r="R14" t="n">
-        <v>38.381</v>
+        <v>38.402</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>cube14_cluster0</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>102</v>
+      </c>
+      <c r="C15" t="n">
+        <v>37</v>
+      </c>
+      <c r="D15" t="n">
+        <v>30</v>
+      </c>
+      <c r="E15" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="H15" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2.4026</v>
+      </c>
+      <c r="J15" t="n">
+        <v>34.8824</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4.2353</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1.7941</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.5784</v>
+      </c>
+      <c r="N15" t="n">
+        <v>8.573499999999999</v>
+      </c>
+      <c r="O15" t="n">
+        <v>3.2647</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3136.902</v>
+      </c>
+      <c r="R15" t="n">
+        <v>38.0098</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cube1_cluster0</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>177</v>
+      </c>
+      <c r="C16" t="n">
+        <v>64</v>
+      </c>
+      <c r="D16" t="n">
+        <v>52</v>
+      </c>
+      <c r="E16" t="n">
+        <v>61</v>
+      </c>
+      <c r="F16" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.4222</v>
+      </c>
+      <c r="J16" t="n">
+        <v>35.7327</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5.5819</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.452</v>
+      </c>
+      <c r="M16" t="n">
+        <v>8.350300000000001</v>
+      </c>
+      <c r="N16" t="n">
+        <v>10.3141</v>
+      </c>
+      <c r="O16" t="n">
+        <v>3.9764</v>
+      </c>
+      <c r="P16" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>3449.5028</v>
+      </c>
+      <c r="R16" t="n">
+        <v>38.2696</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cube37_cluster0</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>93</v>
+      </c>
+      <c r="C17" t="n">
+        <v>27</v>
+      </c>
+      <c r="D17" t="n">
+        <v>34</v>
+      </c>
+      <c r="E17" t="n">
+        <v>32</v>
+      </c>
+      <c r="F17" t="n">
+        <v>29</v>
+      </c>
+      <c r="G17" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.4252</v>
+      </c>
+      <c r="J17" t="n">
+        <v>32.8283</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5.7957</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10.2366</v>
+      </c>
+      <c r="N17" t="n">
+        <v>10.2957</v>
+      </c>
+      <c r="O17" t="n">
+        <v>3.9997</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3351.6237</v>
+      </c>
+      <c r="R17" t="n">
+        <v>38.9724</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>cube5_cluster0</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B18" t="n">
+        <v>75</v>
+      </c>
+      <c r="C18" t="n">
+        <v>29</v>
+      </c>
+      <c r="D18" t="n">
+        <v>19</v>
+      </c>
+      <c r="E18" t="n">
+        <v>27</v>
+      </c>
+      <c r="F18" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G18" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="H18" t="n">
+        <v>36</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2.4523</v>
+      </c>
+      <c r="J18" t="n">
+        <v>37.3595</v>
+      </c>
+      <c r="K18" t="n">
+        <v>6.4133</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>7.4267</v>
+      </c>
+      <c r="N18" t="n">
+        <v>11.1187</v>
+      </c>
+      <c r="O18" t="n">
+        <v>4.2501</v>
+      </c>
+      <c r="P18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3276.7733</v>
+      </c>
+      <c r="R18" t="n">
+        <v>38.4648</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cube16_cluster0</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>122</v>
+      </c>
+      <c r="C19" t="n">
+        <v>36</v>
+      </c>
+      <c r="D19" t="n">
+        <v>46</v>
+      </c>
+      <c r="E19" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="H19" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2.4533</v>
+      </c>
+      <c r="J19" t="n">
+        <v>32.041</v>
+      </c>
+      <c r="K19" t="n">
+        <v>4.1066</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1.7623</v>
+      </c>
+      <c r="N19" t="n">
+        <v>11.8566</v>
+      </c>
+      <c r="O19" t="n">
+        <v>4.567</v>
+      </c>
+      <c r="P19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>3371.4754</v>
+      </c>
+      <c r="R19" t="n">
+        <v>39</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cube20_cluster0</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>102</v>
+      </c>
+      <c r="C20" t="n">
+        <v>36</v>
+      </c>
+      <c r="D20" t="n">
+        <v>32</v>
+      </c>
+      <c r="E20" t="n">
+        <v>34</v>
+      </c>
+      <c r="F20" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="G20" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.4662</v>
+      </c>
+      <c r="J20" t="n">
+        <v>35.3418</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5.9804</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.9706</v>
+      </c>
+      <c r="M20" t="n">
+        <v>8.5784</v>
+      </c>
+      <c r="N20" t="n">
+        <v>9.4147</v>
+      </c>
+      <c r="O20" t="n">
+        <v>3.5904</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>3197.9314</v>
+      </c>
+      <c r="R20" t="n">
+        <v>37.7941</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cube29_cluster0</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>161</v>
+      </c>
+      <c r="C21" t="n">
+        <v>54</v>
+      </c>
+      <c r="D21" t="n">
+        <v>51</v>
+      </c>
+      <c r="E21" t="n">
+        <v>56</v>
+      </c>
+      <c r="F21" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2.4735</v>
+      </c>
+      <c r="J21" t="n">
+        <v>34.9938</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5.9255</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1.0994</v>
+      </c>
+      <c r="M21" t="n">
+        <v>9.1242</v>
+      </c>
+      <c r="N21" t="n">
+        <v>9.6416</v>
+      </c>
+      <c r="O21" t="n">
+        <v>3.7263</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>3092.6832</v>
+      </c>
+      <c r="R21" t="n">
+        <v>38.0018</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cube30_cluster0</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>154</v>
+      </c>
+      <c r="C22" t="n">
+        <v>49</v>
+      </c>
+      <c r="D22" t="n">
+        <v>51</v>
+      </c>
+      <c r="E22" t="n">
+        <v>54</v>
+      </c>
+      <c r="F22" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G22" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.4789</v>
+      </c>
+      <c r="J22" t="n">
+        <v>33.863</v>
+      </c>
+      <c r="K22" t="n">
+        <v>6.2338</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>7.2078</v>
+      </c>
+      <c r="N22" t="n">
+        <v>10.8896</v>
+      </c>
+      <c r="O22" t="n">
+        <v>4.198</v>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>3191.5974</v>
+      </c>
+      <c r="R22" t="n">
+        <v>38.5445</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cube28_cluster0</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>207</v>
+      </c>
+      <c r="C23" t="n">
+        <v>60</v>
+      </c>
+      <c r="D23" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" t="n">
+        <v>72</v>
+      </c>
+      <c r="F23" t="n">
+        <v>29</v>
+      </c>
+      <c r="G23" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2.5064</v>
+      </c>
+      <c r="J23" t="n">
+        <v>33.985</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5.3961</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1.4928</v>
+      </c>
+      <c r="M23" t="n">
+        <v>9.705299999999999</v>
+      </c>
+      <c r="N23" t="n">
+        <v>10.0758</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3.8699</v>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>3260.1111</v>
+      </c>
+      <c r="R23" t="n">
+        <v>38.0759</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cube27_cluster0</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>255</v>
+      </c>
+      <c r="C24" t="n">
+        <v>81</v>
+      </c>
+      <c r="D24" t="n">
+        <v>86</v>
+      </c>
+      <c r="E24" t="n">
+        <v>88</v>
+      </c>
+      <c r="F24" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="H24" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2.5237</v>
+      </c>
+      <c r="J24" t="n">
+        <v>33.8383</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4.8118</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.0588</v>
+      </c>
+      <c r="M24" t="n">
+        <v>8.635300000000001</v>
+      </c>
+      <c r="N24" t="n">
+        <v>9.7125</v>
+      </c>
+      <c r="O24" t="n">
+        <v>3.7543</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>3364.0118</v>
+      </c>
+      <c r="R24" t="n">
+        <v>38.3832</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cube26_cluster0</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>160</v>
+      </c>
+      <c r="C25" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" t="n">
+        <v>55</v>
+      </c>
+      <c r="F25" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G25" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="H25" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="I25" t="n">
+        <v>2.527</v>
+      </c>
+      <c r="J25" t="n">
+        <v>33.7806</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4.2188</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.4062</v>
+      </c>
+      <c r="M25" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="O25" t="n">
+        <v>3.8632</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>3402.25</v>
+      </c>
+      <c r="R25" t="n">
+        <v>38.5429</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cube21_cluster0</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>68</v>
+      </c>
+      <c r="C26" t="n">
+        <v>27</v>
+      </c>
+      <c r="D26" t="n">
+        <v>17</v>
+      </c>
+      <c r="E26" t="n">
+        <v>24</v>
+      </c>
+      <c r="F26" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.5397</v>
+      </c>
+      <c r="J26" t="n">
+        <v>37.9553</v>
+      </c>
+      <c r="K26" t="n">
+        <v>6.1029</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1.2353</v>
+      </c>
+      <c r="M26" t="n">
+        <v>7.6029</v>
+      </c>
+      <c r="N26" t="n">
+        <v>8.7471</v>
+      </c>
+      <c r="O26" t="n">
+        <v>3.3522</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>2738.5441</v>
+      </c>
+      <c r="R26" t="n">
+        <v>36.6744</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cube19_cluster0</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>183</v>
+      </c>
+      <c r="C27" t="n">
+        <v>62</v>
+      </c>
+      <c r="D27" t="n">
+        <v>54</v>
+      </c>
+      <c r="E27" t="n">
+        <v>67</v>
+      </c>
+      <c r="F27" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="G27" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.6249</v>
+      </c>
+      <c r="J27" t="n">
+        <v>35.3156</v>
+      </c>
+      <c r="K27" t="n">
+        <v>5.2896</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2.459</v>
+      </c>
+      <c r="M27" t="n">
+        <v>9.054600000000001</v>
+      </c>
+      <c r="N27" t="n">
+        <v>9.313700000000001</v>
+      </c>
+      <c r="O27" t="n">
+        <v>3.5844</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>3401.3607</v>
+      </c>
+      <c r="R27" t="n">
+        <v>38.4692</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cube22_cluster0</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>79</v>
+      </c>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" t="n">
+        <v>21</v>
+      </c>
+      <c r="E28" t="n">
+        <v>31</v>
+      </c>
+      <c r="F28" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="G28" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="H28" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.6461</v>
+      </c>
+      <c r="J28" t="n">
+        <v>37.2519</v>
+      </c>
+      <c r="K28" t="n">
+        <v>6.3418</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>7.0506</v>
+      </c>
+      <c r="N28" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="O28" t="n">
+        <v>3.8887</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>3034.9494</v>
+      </c>
+      <c r="R28" t="n">
+        <v>38.0108</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cube15_cluster0</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>106</v>
+      </c>
+      <c r="C29" t="n">
+        <v>29</v>
+      </c>
+      <c r="D29" t="n">
+        <v>37</v>
+      </c>
+      <c r="E29" t="n">
+        <v>40</v>
+      </c>
+      <c r="F29" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="H29" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2.6581</v>
+      </c>
+      <c r="J29" t="n">
+        <v>35.3585</v>
+      </c>
+      <c r="K29" t="n">
+        <v>4.2264</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1.0755</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1.7075</v>
+      </c>
+      <c r="N29" t="n">
+        <v>10.5302</v>
+      </c>
+      <c r="O29" t="n">
+        <v>4.0376</v>
+      </c>
+      <c r="P29" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>3095.1132</v>
+      </c>
+      <c r="R29" t="n">
+        <v>38.2197</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cube0_cluster0</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>100</v>
+      </c>
+      <c r="C30" t="n">
+        <v>35</v>
+      </c>
+      <c r="D30" t="n">
+        <v>24</v>
+      </c>
+      <c r="E30" t="n">
+        <v>41</v>
+      </c>
+      <c r="F30" t="n">
+        <v>35</v>
+      </c>
+      <c r="G30" t="n">
+        <v>24</v>
+      </c>
+      <c r="H30" t="n">
+        <v>41</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2.6741</v>
+      </c>
+      <c r="J30" t="n">
+        <v>36.5877</v>
+      </c>
+      <c r="K30" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="M30" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="N30" t="n">
+        <v>10.045</v>
+      </c>
+      <c r="O30" t="n">
+        <v>3.8583</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>3453.69</v>
+      </c>
+      <c r="R30" t="n">
+        <v>38.1543</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cube33_cluster0</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>90</v>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D31" t="n">
+        <v>28</v>
+      </c>
+      <c r="E31" t="n">
+        <v>32</v>
+      </c>
+      <c r="F31" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2.6846</v>
+      </c>
+      <c r="J31" t="n">
+        <v>35.1556</v>
+      </c>
+      <c r="K31" t="n">
+        <v>4.0778</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1.7556</v>
+      </c>
+      <c r="N31" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="O31" t="n">
+        <v>3.7558</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>3338.3556</v>
+      </c>
+      <c r="R31" t="n">
+        <v>38.0921</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>cube25_cluster0</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>84</v>
+      </c>
+      <c r="C32" t="n">
+        <v>29</v>
+      </c>
+      <c r="D32" t="n">
+        <v>25</v>
+      </c>
+      <c r="E32" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="H32" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.6915</v>
+      </c>
+      <c r="J32" t="n">
+        <v>35.3571</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4.0595</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2.131</v>
+      </c>
+      <c r="M32" t="n">
+        <v>1.7024</v>
+      </c>
+      <c r="N32" t="n">
+        <v>9.723800000000001</v>
+      </c>
+      <c r="O32" t="n">
+        <v>3.7168</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>3424.8095</v>
+      </c>
+      <c r="R32" t="n">
+        <v>38.3776</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>cube31_cluster0</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>24</v>
+      </c>
+      <c r="C33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D33" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" t="n">
+        <v>25</v>
+      </c>
+      <c r="G33" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H33" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I33" t="n">
+        <v>2.6927</v>
+      </c>
+      <c r="J33" t="n">
+        <v>34</v>
+      </c>
+      <c r="K33" t="n">
         <v>4</v>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="L33" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="N33" t="n">
+        <v>11.1375</v>
+      </c>
+      <c r="O33" t="n">
+        <v>4.2503</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>3462.0417</v>
+      </c>
+      <c r="R33" t="n">
+        <v>38.4464</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cube23_cluster0</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>24</v>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" t="n">
+        <v>9</v>
+      </c>
+      <c r="F34" t="n">
+        <v>25</v>
+      </c>
+      <c r="G34" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H34" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2.6927</v>
+      </c>
+      <c r="J34" t="n">
+        <v>34</v>
+      </c>
+      <c r="K34" t="n">
         <v>4</v>
       </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>100</v>
-      </c>
-      <c r="I15" t="n">
-        <v>7.3475</v>
-      </c>
-      <c r="J15" t="n">
-        <v>39.992</v>
-      </c>
-      <c r="K15" t="n">
-        <v>6</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M15" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="N15" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="O15" t="n">
-        <v>4.9168</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="L34" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="N34" t="n">
+        <v>11.1375</v>
+      </c>
+      <c r="O34" t="n">
+        <v>4.2503</v>
+      </c>
+      <c r="P34" t="n">
         <v>1</v>
       </c>
-      <c r="Q15" t="n">
-        <v>3357.5</v>
-      </c>
-      <c r="R15" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="S15" t="inlineStr">
+      <c r="Q34" t="n">
+        <v>3462.0417</v>
+      </c>
+      <c r="R34" t="n">
+        <v>38.4464</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cube36_cluster0</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>137</v>
+      </c>
+      <c r="C35" t="n">
+        <v>30</v>
+      </c>
+      <c r="D35" t="n">
+        <v>52</v>
+      </c>
+      <c r="E35" t="n">
+        <v>55</v>
+      </c>
+      <c r="F35" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="G35" t="n">
+        <v>38</v>
+      </c>
+      <c r="H35" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>2.709</v>
+      </c>
+      <c r="J35" t="n">
+        <v>33.4382</v>
+      </c>
+      <c r="K35" t="n">
+        <v>4.6423</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1.0219</v>
+      </c>
+      <c r="M35" t="n">
+        <v>8.6496</v>
+      </c>
+      <c r="N35" t="n">
+        <v>9.4642</v>
+      </c>
+      <c r="O35" t="n">
+        <v>3.6592</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>3418.4891</v>
+      </c>
+      <c r="R35" t="n">
+        <v>38.5151</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cube6_cluster0</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>137</v>
+      </c>
+      <c r="C36" t="n">
+        <v>40</v>
+      </c>
+      <c r="D36" t="n">
+        <v>40</v>
+      </c>
+      <c r="E36" t="n">
+        <v>57</v>
+      </c>
+      <c r="F36" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G36" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="H36" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2.7291</v>
+      </c>
+      <c r="J36" t="n">
+        <v>36.7866</v>
+      </c>
+      <c r="K36" t="n">
+        <v>5.5182</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2.7591</v>
+      </c>
+      <c r="M36" t="n">
+        <v>5.3796</v>
+      </c>
+      <c r="N36" t="n">
+        <v>9.5219</v>
+      </c>
+      <c r="O36" t="n">
+        <v>3.6725</v>
+      </c>
+      <c r="P36" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>3421.0657</v>
+      </c>
+      <c r="R36" t="n">
+        <v>38.3191</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cube18_cluster0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>99</v>
+      </c>
+      <c r="C37" t="n">
+        <v>35</v>
+      </c>
+      <c r="D37" t="n">
+        <v>25</v>
+      </c>
+      <c r="E37" t="n">
+        <v>39</v>
+      </c>
+      <c r="F37" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="H37" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="I37" t="n">
+        <v>2.736</v>
+      </c>
+      <c r="J37" t="n">
+        <v>36.0596</v>
+      </c>
+      <c r="K37" t="n">
+        <v>4.7677</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2.8586</v>
+      </c>
+      <c r="M37" t="n">
+        <v>9.494899999999999</v>
+      </c>
+      <c r="N37" t="n">
+        <v>9.175800000000001</v>
+      </c>
+      <c r="O37" t="n">
+        <v>3.5627</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>3411.1616</v>
+      </c>
+      <c r="R37" t="n">
+        <v>38.443</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cube32_cluster0</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>67</v>
+      </c>
+      <c r="C38" t="n">
+        <v>23</v>
+      </c>
+      <c r="D38" t="n">
+        <v>18</v>
+      </c>
+      <c r="E38" t="n">
+        <v>26</v>
+      </c>
+      <c r="F38" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="G38" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H38" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2.8128</v>
+      </c>
+      <c r="J38" t="n">
+        <v>37.2239</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4.2537</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.6567</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1.4776</v>
+      </c>
+      <c r="N38" t="n">
+        <v>9.6015</v>
+      </c>
+      <c r="O38" t="n">
+        <v>3.6633</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>3473.3284</v>
+      </c>
+      <c r="R38" t="n">
+        <v>38.2836</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>cube24_cluster0</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>67</v>
+      </c>
+      <c r="C39" t="n">
+        <v>23</v>
+      </c>
+      <c r="D39" t="n">
+        <v>18</v>
+      </c>
+      <c r="E39" t="n">
+        <v>26</v>
+      </c>
+      <c r="F39" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="G39" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H39" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="I39" t="n">
+        <v>2.8128</v>
+      </c>
+      <c r="J39" t="n">
+        <v>37.2239</v>
+      </c>
+      <c r="K39" t="n">
+        <v>4.2537</v>
+      </c>
+      <c r="L39" t="n">
+        <v>2.6567</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1.4776</v>
+      </c>
+      <c r="N39" t="n">
+        <v>9.6015</v>
+      </c>
+      <c r="O39" t="n">
+        <v>3.6633</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>3473.3284</v>
+      </c>
+      <c r="R39" t="n">
+        <v>38.2836</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>cube12_cluster0</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>38</v>
+      </c>
+      <c r="C40" t="n">
+        <v>7</v>
+      </c>
+      <c r="D40" t="n">
+        <v>15</v>
+      </c>
+      <c r="E40" t="n">
+        <v>16</v>
+      </c>
+      <c r="F40" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G40" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H40" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2.8274</v>
+      </c>
+      <c r="J40" t="n">
+        <v>37.3421</v>
+      </c>
+      <c r="K40" t="n">
+        <v>4</v>
+      </c>
+      <c r="L40" t="n">
+        <v>3.2632</v>
+      </c>
+      <c r="M40" t="n">
+        <v>1.3421</v>
+      </c>
+      <c r="N40" t="n">
+        <v>8.763199999999999</v>
+      </c>
+      <c r="O40" t="n">
+        <v>3.4287</v>
+      </c>
+      <c r="P40" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>3409.1316</v>
+      </c>
+      <c r="R40" t="n">
+        <v>38.8233</v>
+      </c>
+      <c r="S40" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
@@ -1407,7 +2982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1452,68 +3027,98 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Total mg/d AF  suple y pan</t>
+          <t>UMAP 2D sobre espacio de features</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>n_cubes</t>
+          <t>umap_n_neighbors</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>overlap</t>
+          <t>umap_min_dist</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dbscan_eps</t>
+          <t>umap_seed</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dbscan_min_samples</t>
+          <t>n_cubes</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nodos</t>
+          <t>overlap</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>dbscan_eps</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dbscan_min_samples</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>nodos</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>aristas</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>5</v>
+      <c r="B13" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>